<commit_message>
feat: expand market analysis workflows
Add portfolio news sentiment, macro reporting updates, and richer AI analysis support so the app can surface broader market context.
</commit_message>
<xml_diff>
--- a/backend/data/macro_daily.xlsx
+++ b/backend/data/macro_daily.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,11 +475,11 @@
         <v>46023</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -496,11 +496,11 @@
         <v>46113</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -517,11 +517,11 @@
         <v>46113</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -538,11 +538,11 @@
         <v>46113</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -559,11 +559,11 @@
         <v>46113</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -580,11 +580,11 @@
         <v>46151</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -601,11 +601,11 @@
         <v>46113</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -622,11 +622,11 @@
         <v>46113</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -643,11 +643,11 @@
         <v>46113</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -664,11 +664,11 @@
         <v>46113</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -679,17 +679,17 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4.47</v>
+        <v>4.59</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -700,17 +700,17 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>4.09</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -721,17 +721,17 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>118.0392</v>
+        <v>119.2825</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>46150</v>
+        <v>46157</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -742,17 +742,17 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.76</v>
+        <v>2.83</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>46156</v>
+        <v>46160</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -769,11 +769,11 @@
         <v>46155</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -790,11 +790,11 @@
         <v>46082</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>
@@ -805,17 +805,17 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.4699999999999998</v>
+        <v>0.5</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>46160.32586234729</v>
+        <v>46161.9563583303</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>46160</v>
+        <v>46161</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-05-18T03:49:14.508558+00:00</t>
+          <t>2026-05-19T18:57:09.361378+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>